<commit_message>
Made the variable definitions donwload default to excel
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\SurveyResults\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614EA0D4-AB7F-4983-9F12-57701C0F1DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="32130" yWindow="3570" windowWidth="19260" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -169,9 +175,6 @@
     <t>The participant's response to "How much experience did you have with VR Gaming before today?"</t>
   </si>
   <si>
-    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 8 and 9, participants saw 4 blocks with 3-4 DMs each (4 in the case of Multi KDMA). The following columns describe each page of the survey using this BX_DMY format.</t>
-  </si>
-  <si>
     <t>The alignment level of the DM based on the alignment gathered from the participant's text responses</t>
   </si>
   <si>
@@ -259,12 +262,6 @@
     <t>Levels</t>
   </si>
   <si>
-    <t>6, 7, 8, 9</t>
-  </si>
-  <si>
-    <r>
-      <t/>
-    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -278,7 +275,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -298,7 +295,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -318,7 +315,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -338,7 +335,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -376,9 +373,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -391,7 +385,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -411,7 +405,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -431,7 +425,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -451,7 +445,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -471,9 +465,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -486,7 +477,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -506,7 +497,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -526,7 +517,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -546,7 +537,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -566,9 +557,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -581,7 +569,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -601,7 +589,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -621,7 +609,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -641,7 +629,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -661,9 +649,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -676,7 +661,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -696,7 +681,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -716,7 +701,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -736,7 +721,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -763,9 +748,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -778,7 +760,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -798,7 +780,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -818,7 +800,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -838,7 +820,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -858,9 +840,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -873,7 +852,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -893,7 +872,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -913,7 +892,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -933,7 +912,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFffffff"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -950,14 +929,19 @@
       </rPr>
       <t xml:space="preserve"> 5 - Completely confident</t>
     </r>
+  </si>
+  <si>
+    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 15, participants saw 5 blocks with 2-3 DMs each (multi-KDMA blocks have aligned and baseline; the single MF block also includes misaligned). The following columns describe each page of the survey using this BX_DMY format.</t>
+  </si>
+  <si>
+    <t>6, 7, 8, 9,10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -976,6 +960,20 @@
       <color rgb="FF212529"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1006,31 +1004,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1041,10 +1042,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -1082,71 +1083,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1174,7 +1175,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1197,11 +1198,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1210,13 +1211,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1226,7 +1227,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1235,7 +1236,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1244,7 +1245,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1252,10 +1253,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1320,58 +1321,39 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AP3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="5" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="5" width="18.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="5" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="5" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="5" width="18.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="5" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="5" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="5" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="1" max="6" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="16" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="18.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="19.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="24.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="22.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="25.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="18.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="23" style="5" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="25" style="5" bestFit="1" customWidth="1"/>
+    <col min="38" max="42" width="32.1796875" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="73.5" customFormat="1" s="1">
+    <row r="1" spans="1:42" s="1" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1499,7 +1481,7 @@
         <v>41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="235.5" customFormat="1" s="1">
+    <row r="2" spans="1:42" s="1" customFormat="1" ht="235.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>42</v>
       </c>
@@ -1531,107 +1513,107 @@
         <v>50</v>
       </c>
       <c r="K2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="W2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="W2" s="2" t="s">
+      <c r="X2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="X2" s="2" t="s">
+      <c r="Y2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Y2" s="2" t="s">
+      <c r="Z2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Z2" s="2" t="s">
+      <c r="AA2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AA2" s="2" t="s">
+      <c r="AB2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AC2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AC2" s="2" t="s">
+      <c r="AD2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AE2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AG2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AH2" s="2" t="s">
+      <c r="AI2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AI2" s="2" t="s">
+      <c r="AJ2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AJ2" s="2" t="s">
+      <c r="AK2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AK2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL2" s="2" t="s">
+      <c r="AM2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AM2" s="2" t="s">
+      <c r="AN2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="AN2" s="2" t="s">
+      <c r="AO2" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AO2" s="2" t="s">
+      <c r="AP2" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:42" s="1" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="AP2" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="195" customFormat="1" s="1">
-      <c r="A3" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
@@ -1640,39 +1622,39 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
       <c r="R3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="T3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="U3" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="W3" s="2"/>
       <c r="X3" s="2"/>
@@ -1682,28 +1664,28 @@
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
       <c r="AD3" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="AE3" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AJ3" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="AJ3" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="AK3" s="2"/>
       <c r="AL3" s="2"/>
       <c r="AM3" s="2"/>
       <c r="AN3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AO3" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="AO3" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="AP3" s="2"/>
     </row>

</xml_diff>

<commit_message>
Updated variable defs columns for ph2
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\SurveyResults\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614EA0D4-AB7F-4983-9F12-57701C0F1DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFA0444-7FBB-4162-8EF3-55738B6B0DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32130" yWindow="3570" windowWidth="19260" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="103">
   <si>
     <t>Variables</t>
   </si>
@@ -226,9 +226,6 @@
     <t>The response to the first forced choice question (aligned vs baseline, or follow the previous column for Multi KDMA)</t>
   </si>
   <si>
-    <t>The response to ""For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the first forced choice</t>
-  </si>
-  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the first forced choice</t>
   </si>
   <si>
@@ -241,9 +238,6 @@
     <t>The response to the second forced choice question (aligned vs misaligned, or follow the previous column for Multi KDMA)</t>
   </si>
   <si>
-    <t>The response to ""For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the second forced choice</t>
-  </si>
-  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the second forced choice question</t>
   </si>
   <si>
@@ -251,9 +245,6 @@
   </si>
   <si>
     <t>The response to the third forced choice question (follow the previous column)</t>
-  </si>
-  <si>
-    <t>The response to ""For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the third forced choice</t>
   </si>
   <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the third forced choice question</t>
@@ -935,6 +926,36 @@
   </si>
   <si>
     <t>6, 7, 8, 9,10</t>
+  </si>
+  <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the second forced choice</t>
+  </si>
+  <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the third forced choice</t>
+  </si>
+  <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the first forced choice</t>
+  </si>
+  <si>
+    <t>VR Comfort Level</t>
+  </si>
+  <si>
+    <t>The participant's response to "After completing the VR experience, my current physical state is..."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very Comfortable, Slightly Uncomfortable, Neutral, Comfortable, Very Comfortable </t>
+  </si>
+  <si>
+    <t>BX_Compare_Time (mm:ss)</t>
+  </si>
+  <si>
+    <t>The amount of time the participant spent (Minutes:Seconds) on the comparison page</t>
+  </si>
+  <si>
+    <t>BX_Compare_FC4-6</t>
+  </si>
+  <si>
+    <t>The response to the fourth - sixth forced choice question (follow the previous column). Exclusive to the September Evaluation</t>
   </si>
 </sst>
 </file>
@@ -1325,35 +1346,40 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AP3"/>
+  <dimension ref="A1:AS3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="6" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.453125" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="16" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.81640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="18.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="19.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="24.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="22.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="25.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="18.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="23" style="5" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="25" style="5" bestFit="1" customWidth="1"/>
-    <col min="38" max="42" width="32.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.7265625" style="5" customWidth="1"/>
+    <col min="12" max="17" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="18.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.453125" style="5" customWidth="1"/>
+    <col min="30" max="30" width="19.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="24.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="22.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="25.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="18.26953125" style="5" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="23" style="5" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="25" style="5" bestFit="1" customWidth="1"/>
+    <col min="40" max="44" width="32.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="24.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" s="1" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:45" s="1" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1385,103 +1411,112 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="AD1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>41</v>
       </c>
+      <c r="AS1" s="1" t="s">
+        <v>101</v>
+      </c>
     </row>
-    <row r="2" spans="1:42" s="1" customFormat="1" ht="235.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:45" s="1" customFormat="1" ht="235.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>42</v>
       </c>
@@ -1513,107 +1548,116 @@
         <v>50</v>
       </c>
       <c r="K2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AH2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AN2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AP2" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AQ2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="AR2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AF2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AG2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AH2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AI2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="AJ2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="AM2" s="2" t="s">
+      <c r="AS2" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:45" s="1" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="AN2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="AO2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="AP2" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:42" s="1" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
@@ -1622,72 +1666,76 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="O3" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="T3" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="U3" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="W3" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="T3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="W3" s="2"/>
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
-      <c r="AD3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE3" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="AF3" s="2"/>
-      <c r="AG3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AG3" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="AH3" s="2"/>
-      <c r="AI3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AJ3" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="AK3" s="2"/>
-      <c r="AL3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
+      <c r="AK3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AL3" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="AM3" s="2"/>
-      <c r="AN3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AO3" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="AP3" s="2"/>
+      <c r="AN3" s="2"/>
+      <c r="AO3" s="2"/>
+      <c r="AP3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AR3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
var defs, quote typo
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\SurveyResults\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFA0444-7FBB-4162-8EF3-55738B6B0DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="113">
   <si>
     <t>Variables</t>
   </si>
@@ -52,6 +46,9 @@
     <t>VR Experience Level</t>
   </si>
   <si>
+    <t>VR Comfort Level</t>
+  </si>
+  <si>
     <t>BX_DMY</t>
   </si>
   <si>
@@ -67,6 +64,12 @@
     <t>BX_DM1_Name</t>
   </si>
   <si>
+    <t>BX_DMY_ADMName</t>
+  </si>
+  <si>
+    <t>BX_DMY_Subpop</t>
+  </si>
+  <si>
     <t>BX_DMY_Time</t>
   </si>
   <si>
@@ -88,6 +91,12 @@
     <t>BX_DMY_Trust</t>
   </si>
   <si>
+    <t>BX_DMY_Distrust</t>
+  </si>
+  <si>
+    <t>BX_DMY_Trustworthy(BEN)</t>
+  </si>
+  <si>
     <t>BX_Compare_DM1</t>
   </si>
   <si>
@@ -103,6 +112,9 @@
     <t>BX_Compare_Time</t>
   </si>
   <si>
+    <t>BX_Compare_Time (mm:ss)</t>
+  </si>
+  <si>
     <t>BX_Compare_FC1_Alignment</t>
   </si>
   <si>
@@ -148,6 +160,9 @@
     <t>BX_Compare_FC3_Explain</t>
   </si>
   <si>
+    <t>BX_Compare_FC4-6</t>
+  </si>
+  <si>
     <t>Definition</t>
   </si>
   <si>
@@ -175,6 +190,12 @@
     <t>The participant's response to "How much experience did you have with VR Gaming before today?"</t>
   </si>
   <si>
+    <t>The participant's response to "After completing the VR experience, my current physical state is..."</t>
+  </si>
+  <si>
+    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 15, participants saw 5 blocks with 2-3 DMs each (multi-KDMA blocks have aligned and baseline; the single MF block also includes misaligned). The following columns describe each page of the survey using this BX_DMY format.</t>
+  </si>
+  <si>
     <t>The alignment level of the DM based on the alignment gathered from the participant's text responses</t>
   </si>
   <si>
@@ -184,6 +205,12 @@
     <t>The name assigned to the DM the participant viewed.</t>
   </si>
   <si>
+    <t>The model of the observed adm</t>
+  </si>
+  <si>
+    <t>Subpopulation group of the observed ADM. Only applies to Oracle.</t>
+  </si>
+  <si>
     <t>The time (minutes) the participant spent on this page</t>
   </si>
   <si>
@@ -205,6 +232,12 @@
     <t>The participant's response to "I would be comfortable allowing this medic to execute medical triage, even if I could not monitor it"</t>
   </si>
   <si>
+    <t>“Based on this experience, I cannot rely on this person with complete confidence.”</t>
+  </si>
+  <si>
+    <t>"This medic really looks out for what is important to me.”</t>
+  </si>
+  <si>
     <t>The name and alignment value of the first medic being compared in this comparison page</t>
   </si>
   <si>
@@ -220,12 +253,18 @@
     <t>The amount of time the participant spent (Minutes) on the comparison page</t>
   </si>
   <si>
+    <t>The amount of time the participant spent (Minutes:Seconds) on the comparison page</t>
+  </si>
+  <si>
     <t>The alignment of the first two DMs being compared</t>
   </si>
   <si>
     <t>The response to the first forced choice question (aligned vs baseline, or follow the previous column for Multi KDMA)</t>
   </si>
   <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the first forced choice</t>
+  </si>
+  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the first forced choice</t>
   </si>
   <si>
@@ -238,6 +277,9 @@
     <t>The response to the second forced choice question (aligned vs misaligned, or follow the previous column for Multi KDMA)</t>
   </si>
   <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the second forced choice</t>
+  </si>
+  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the second forced choice question</t>
   </si>
   <si>
@@ -247,12 +289,24 @@
     <t>The response to the third forced choice question (follow the previous column)</t>
   </si>
   <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the third forced choice</t>
+  </si>
+  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the third forced choice question</t>
   </si>
   <si>
+    <t>The response to the fourth - sixth forced choice question (follow the previous column). Exclusive to the September Evaluation</t>
+  </si>
+  <si>
     <t>Levels</t>
   </si>
   <si>
+    <t>6, 7, 8, 9, 10, 11</t>
+  </si>
+  <si>
+    <r>
+      <t/>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -266,7 +320,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -286,7 +340,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -306,7 +360,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -326,7 +380,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -345,6 +399,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Very Comfortable, Slightly Uncomfortable, Neutral, Comfortable, Very Comfortable </t>
+  </si>
+  <si>
     <t>B1_DM1, B1_DM2, B1_DM3, B1_DM4, B2_DM1, B2_DM2, etc.</t>
   </si>
   <si>
@@ -360,10 +417,19 @@
     <t>Medic-LN, where L is a letter and N is a number</t>
   </si>
   <si>
+    <t xml:space="preserve">e.g Oracle, ALIGN-ADM-Ph2-DirectRegression-BertRelevance-Mistral-7B-Instruct-v0.3_01_12, etc. </t>
+  </si>
+  <si>
+    <t>A, B</t>
+  </si>
+  <si>
     <t xml:space="preserve">1-3 </t>
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -376,7 +442,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -396,7 +462,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -416,7 +482,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -436,7 +502,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -456,6 +522,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -468,7 +537,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -488,7 +557,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -508,7 +577,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -528,7 +597,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -548,6 +617,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -560,7 +632,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -580,7 +652,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -600,7 +672,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -620,7 +692,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -640,6 +712,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -652,7 +727,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -672,7 +747,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -692,7 +767,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -712,7 +787,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -739,6 +814,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -751,7 +829,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -771,7 +849,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -791,7 +869,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -811,7 +889,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -831,6 +909,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -843,7 +924,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -863,7 +944,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -883,7 +964,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -903,7 +984,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -920,49 +1001,14 @@
       </rPr>
       <t xml:space="preserve"> 5 - Completely confident</t>
     </r>
-  </si>
-  <si>
-    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 15, participants saw 5 blocks with 2-3 DMs each (multi-KDMA blocks have aligned and baseline; the single MF block also includes misaligned). The following columns describe each page of the survey using this BX_DMY format.</t>
-  </si>
-  <si>
-    <t>6, 7, 8, 9,10</t>
-  </si>
-  <si>
-    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the second forced choice</t>
-  </si>
-  <si>
-    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the third forced choice</t>
-  </si>
-  <si>
-    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the first forced choice</t>
-  </si>
-  <si>
-    <t>VR Comfort Level</t>
-  </si>
-  <si>
-    <t>The participant's response to "After completing the VR experience, my current physical state is..."</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very Comfortable, Slightly Uncomfortable, Neutral, Comfortable, Very Comfortable </t>
-  </si>
-  <si>
-    <t>BX_Compare_Time (mm:ss)</t>
-  </si>
-  <si>
-    <t>The amount of time the participant spent (Minutes:Seconds) on the comparison page</t>
-  </si>
-  <si>
-    <t>BX_Compare_FC4-6</t>
-  </si>
-  <si>
-    <t>The response to the fourth - sixth forced choice question (follow the previous column). Exclusive to the September Evaluation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -978,23 +1024,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF212529"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF212529"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1024,35 +1062,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="10">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1063,10 +1110,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -1104,71 +1151,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1196,7 +1243,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1219,11 +1266,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1232,13 +1279,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1248,7 +1295,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1257,7 +1304,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1266,7 +1313,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1274,10 +1321,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1342,44 +1389,65 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AS3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AW3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.7265625" style="5" customWidth="1"/>
-    <col min="12" max="17" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.81640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="18.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.453125" style="5" customWidth="1"/>
-    <col min="30" max="30" width="19.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="24.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="22.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="25.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="18.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="23" style="5" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="25" style="5" bestFit="1" customWidth="1"/>
-    <col min="40" max="44" width="32.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="24.453125" customWidth="1"/>
+    <col min="1" max="1" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="8" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="8" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="7" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="7" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="8" width="16.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="8" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="7" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="7" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="7" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="7" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="7" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="7" width="22.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="7" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="7" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="7" width="18.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="7" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="7" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="7" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="9" width="24.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" s="1" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1411,331 +1479,368 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="S1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="Z1" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="AA1" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AC1" s="2" t="s">
-        <v>99</v>
+        <v>28</v>
       </c>
       <c r="AD1" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AF1" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="AO1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AP1" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="AQ1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="AR1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>101</v>
+        <v>43</v>
+      </c>
+      <c r="AS1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="4" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:45" s="1" customFormat="1" ht="235.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="289.5" customFormat="1" s="1">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>64</v>
+        <v>71</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AD2" s="2" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="AG2" s="2" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="AH2" s="2" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="AI2" s="2" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="AJ2" s="2" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="AK2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AM2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AN2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AO2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AP2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AT2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AU2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="AV2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AW2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="AL2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AM2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AN2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="AO2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AP2" s="2" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="262.5" customFormat="1" s="1">
+      <c r="A3" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="AQ2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="AR2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS2" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:45" s="1" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="3"/>
+      <c r="E3" s="5"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="K3" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="M3" s="2" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>81</v>
+        <v>100</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>84</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
       <c r="U3" s="2" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z3" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
-      <c r="AF3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AG3" s="2" t="s">
-        <v>89</v>
-      </c>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
-      <c r="AJ3" s="2"/>
+      <c r="AJ3" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="AK3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AL3" s="2" t="s">
-        <v>90</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="AL3" s="2"/>
       <c r="AM3" s="2"/>
       <c r="AN3" s="2"/>
-      <c r="AO3" s="2"/>
+      <c r="AO3" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="AP3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AQ3" s="2" t="s">
-        <v>90</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="AQ3" s="2"/>
       <c r="AR3" s="2"/>
+      <c r="AS3" s="2"/>
+      <c r="AT3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AU3" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="AV3" s="2"/>
+      <c r="AW3" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
ITM-1333: Survey Results Update and Table Virtualization (#461)
* large refactor

* new gql endpoint

* use new end

* almost there

* comp scores visible

* header update and new rating metrics

* Delegation Preference

* exempt

* demo data fallback

* lookup fixes

* var defs

* def format

* table virtualization optimize

* rq1 bug, styling, optomize

* eval 16

* clean up

* var defs, quote typo

* should be done

* merge conflict error
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\SurveyResults\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFA0444-7FBB-4162-8EF3-55738B6B0DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="115">
   <si>
     <t>Variables</t>
   </si>
@@ -52,6 +46,9 @@
     <t>VR Experience Level</t>
   </si>
   <si>
+    <t>VR Comfort Level</t>
+  </si>
+  <si>
     <t>BX_DMY</t>
   </si>
   <si>
@@ -67,6 +64,12 @@
     <t>BX_DM1_Name</t>
   </si>
   <si>
+    <t>BX_DMY_ADMName</t>
+  </si>
+  <si>
+    <t>BX_DMY_Subpop</t>
+  </si>
+  <si>
     <t>BX_DMY_Time</t>
   </si>
   <si>
@@ -88,6 +91,15 @@
     <t>BX_DMY_Trust</t>
   </si>
   <si>
+    <t>BX_DMY_Distrust</t>
+  </si>
+  <si>
+    <t>BX_DMY_Trustworthy(INT)</t>
+  </si>
+  <si>
+    <t>BX_DMY_Trustworthy(BEN)</t>
+  </si>
+  <si>
     <t>BX_Compare_DM1</t>
   </si>
   <si>
@@ -103,6 +115,9 @@
     <t>BX_Compare_Time</t>
   </si>
   <si>
+    <t>BX_Compare_Time (mm:ss)</t>
+  </si>
+  <si>
     <t>BX_Compare_FC1_Alignment</t>
   </si>
   <si>
@@ -148,6 +163,9 @@
     <t>BX_Compare_FC3_Explain</t>
   </si>
   <si>
+    <t>BX_Compare_FC4-6</t>
+  </si>
+  <si>
     <t>Definition</t>
   </si>
   <si>
@@ -175,6 +193,12 @@
     <t>The participant's response to "How much experience did you have with VR Gaming before today?"</t>
   </si>
   <si>
+    <t>The participant's response to "After completing the VR experience, my current physical state is..."</t>
+  </si>
+  <si>
+    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 15, participants saw 5 blocks with 2-3 DMs each (multi-KDMA blocks have aligned and baseline; the single MF block also includes misaligned). The following columns describe each page of the survey using this BX_DMY format.</t>
+  </si>
+  <si>
     <t>The alignment level of the DM based on the alignment gathered from the participant's text responses</t>
   </si>
   <si>
@@ -184,6 +208,12 @@
     <t>The name assigned to the DM the participant viewed.</t>
   </si>
   <si>
+    <t>The model of the observed adm</t>
+  </si>
+  <si>
+    <t>Subpopulation group of the observed ADM. Only applies to Oracle.</t>
+  </si>
+  <si>
     <t>The time (minutes) the participant spent on this page</t>
   </si>
   <si>
@@ -205,6 +235,15 @@
     <t>The participant's response to "I would be comfortable allowing this medic to execute medical triage, even if I could not monitor it"</t>
   </si>
   <si>
+    <t>“Based on this experience, I cannot rely on this person with complete confidence.”</t>
+  </si>
+  <si>
+    <t>“This medic’s actions and behaviors are not very consistent.”</t>
+  </si>
+  <si>
+    <t>"This medic really looks out for what is important to me.”</t>
+  </si>
+  <si>
     <t>The name and alignment value of the first medic being compared in this comparison page</t>
   </si>
   <si>
@@ -220,12 +259,18 @@
     <t>The amount of time the participant spent (Minutes) on the comparison page</t>
   </si>
   <si>
+    <t>The amount of time the participant spent (Minutes:Seconds) on the comparison page</t>
+  </si>
+  <si>
     <t>The alignment of the first two DMs being compared</t>
   </si>
   <si>
     <t>The response to the first forced choice question (aligned vs baseline, or follow the previous column for Multi KDMA)</t>
   </si>
   <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the first forced choice</t>
+  </si>
+  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the first forced choice</t>
   </si>
   <si>
@@ -238,6 +283,9 @@
     <t>The response to the second forced choice question (aligned vs misaligned, or follow the previous column for Multi KDMA)</t>
   </si>
   <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the second forced choice</t>
+  </si>
+  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the second forced choice question</t>
   </si>
   <si>
@@ -247,12 +295,24 @@
     <t>The response to the third forced choice question (follow the previous column)</t>
   </si>
   <si>
+    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the third forced choice</t>
+  </si>
+  <si>
     <t>The response to "Rate your confidence about the delegation decision indicated in the previous question" for the third forced choice question</t>
   </si>
   <si>
+    <t>The response to the fourth - sixth forced choice question (follow the previous column). Exclusive to the September Evaluation</t>
+  </si>
+  <si>
     <t>Levels</t>
   </si>
   <si>
+    <t>6, 7, 8, 9, 10, 11</t>
+  </si>
+  <si>
+    <r>
+      <t/>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -266,7 +326,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -286,7 +346,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -306,7 +366,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -326,7 +386,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -345,6 +405,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Very Comfortable, Slightly Uncomfortable, Neutral, Comfortable, Very Comfortable </t>
+  </si>
+  <si>
     <t>B1_DM1, B1_DM2, B1_DM3, B1_DM4, B2_DM1, B2_DM2, etc.</t>
   </si>
   <si>
@@ -360,10 +423,19 @@
     <t>Medic-LN, where L is a letter and N is a number</t>
   </si>
   <si>
+    <t xml:space="preserve">e.g Oracle, ALIGN-ADM-Ph2-DirectRegression-BertRelevance-Mistral-7B-Instruct-v0.3_01_12, etc. </t>
+  </si>
+  <si>
+    <t>A, B</t>
+  </si>
+  <si>
     <t xml:space="preserve">1-3 </t>
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -376,7 +448,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -396,7 +468,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -416,7 +488,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -436,7 +508,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -456,6 +528,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -468,7 +543,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -488,7 +563,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -508,7 +583,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -528,7 +603,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -548,6 +623,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -560,7 +638,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -580,7 +658,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -600,7 +678,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -620,7 +698,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -640,6 +718,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -652,7 +733,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -672,7 +753,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -692,7 +773,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -712,7 +793,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -739,6 +820,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -751,7 +835,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -771,7 +855,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -791,7 +875,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -811,7 +895,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -831,6 +915,9 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -843,7 +930,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -863,7 +950,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -883,7 +970,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -903,7 +990,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FFffffff"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -920,49 +1007,14 @@
       </rPr>
       <t xml:space="preserve"> 5 - Completely confident</t>
     </r>
-  </si>
-  <si>
-    <t>X refers to the block number, Y refers to the DM number the participant saw. For Eval 15, participants saw 5 blocks with 2-3 DMs each (multi-KDMA blocks have aligned and baseline; the single MF block also includes misaligned). The following columns describe each page of the survey using this BX_DMY format.</t>
-  </si>
-  <si>
-    <t>6, 7, 8, 9,10</t>
-  </si>
-  <si>
-    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the second forced choice</t>
-  </si>
-  <si>
-    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the third forced choice</t>
-  </si>
-  <si>
-    <t>The response to "For a set of future patients, you can delegate the patients to either or both of these decision-makers. In this scenario, either of these decision makers could handle 100% of this task load in a timely manner and it is not more or less efficient to divide the work between them. How would you allocate the patients between these two decision makers?" for the first forced choice</t>
-  </si>
-  <si>
-    <t>VR Comfort Level</t>
-  </si>
-  <si>
-    <t>The participant's response to "After completing the VR experience, my current physical state is..."</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very Comfortable, Slightly Uncomfortable, Neutral, Comfortable, Very Comfortable </t>
-  </si>
-  <si>
-    <t>BX_Compare_Time (mm:ss)</t>
-  </si>
-  <si>
-    <t>The amount of time the participant spent (Minutes:Seconds) on the comparison page</t>
-  </si>
-  <si>
-    <t>BX_Compare_FC4-6</t>
-  </si>
-  <si>
-    <t>The response to the fourth - sixth forced choice question (follow the previous column). Exclusive to the September Evaluation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -978,23 +1030,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF212529"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF212529"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1024,35 +1068,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="10">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1063,10 +1116,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -1104,71 +1157,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1196,7 +1249,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1219,11 +1272,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1232,13 +1285,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1248,7 +1301,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1257,7 +1310,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1266,7 +1319,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1274,10 +1327,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1342,44 +1395,66 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AS3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AX3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.7265625" style="5" customWidth="1"/>
-    <col min="12" max="17" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.81640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="18.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.453125" style="5" customWidth="1"/>
-    <col min="30" max="30" width="19.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="24.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="22.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="25.7265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="18.26953125" style="5" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="23" style="5" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="25" style="5" bestFit="1" customWidth="1"/>
-    <col min="40" max="44" width="32.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="24.453125" customWidth="1"/>
+    <col min="1" max="1" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="8" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="8" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="7" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="7" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="8" width="16.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="8" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="8" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="7" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="7" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="7" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="7" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="7" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="7" width="22.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="7" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="7" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="7" width="18.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="7" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="7" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="7" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="50" max="50" style="9" width="24.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" s="1" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1411,331 +1486,377 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="S1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="Z1" s="3" t="s">
         <v>25</v>
       </c>
+      <c r="AA1" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="AB1" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AC1" s="2" t="s">
-        <v>99</v>
+        <v>28</v>
       </c>
       <c r="AD1" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AF1" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="AO1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AP1" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="AQ1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="AR1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>101</v>
+        <v>43</v>
+      </c>
+      <c r="AS1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:45" s="1" customFormat="1" ht="235.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="289.5" customFormat="1" s="1">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>65</v>
+        <v>72</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="AD2" s="2" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="AF2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="AH2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="AK2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AM2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AN2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AO2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AP2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AQ2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AR2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AS2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AT2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="AU2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AV2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AW2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AX2" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="AG2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AH2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AI2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AJ2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AK2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="AL2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AM2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AN2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="AO2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AP2" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AQ2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="AR2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AS2" s="1" t="s">
-        <v>102</v>
-      </c>
     </row>
-    <row r="3" spans="1:45" s="1" customFormat="1" ht="195" customHeight="1" x14ac:dyDescent="0.35">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="262.5" customFormat="1" s="1">
       <c r="A3" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="3"/>
+      <c r="E3" s="5"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>81</v>
+        <v>102</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>84</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
       <c r="U3" s="2" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="2"/>
+        <v>109</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="Z3" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>111</v>
+      </c>
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
-      <c r="AF3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AG3" s="2" t="s">
-        <v>89</v>
-      </c>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
       <c r="AK3" s="2" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="AL3" s="2" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="AM3" s="2"/>
       <c r="AN3" s="2"/>
       <c r="AO3" s="2"/>
       <c r="AP3" s="2" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="AQ3" s="2" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="AR3" s="2"/>
+      <c r="AS3" s="2"/>
+      <c r="AT3" s="2"/>
+      <c r="AU3" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="AV3" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="AW3" s="2"/>
+      <c r="AX3" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Itm 1413: /survey-results update (#503)
* initial change

* improve query

* targets printed out in full

* var def

* clean up super ugly signature

* fixed conflicting css for virtualized vs non-virtualized tables. Removed weird empty row bug

* eval 15 attr and ps-af target fix
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
@@ -307,7 +307,7 @@
     <t>Levels</t>
   </si>
   <si>
-    <t>6, 7, 8, 9, 10, 11</t>
+    <t>6, 7, 8, 9, 10, 11, 12</t>
   </si>
   <si>
     <r>
@@ -1068,16 +1068,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1090,9 +1087,6 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general" wrapText="1"/>
@@ -1402,56 +1396,56 @@
   <dimension ref="A1:AX3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="8" width="14.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="8" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="7" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="7" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="8" width="16.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="8" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="8" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="7" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="7" width="18.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="7" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="7" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="7" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="7" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="7" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="7" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="7" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="7" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="7" width="18.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="7" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="43" max="43" style="7" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="44" max="44" style="7" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="45" max="45" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="46" max="46" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="47" max="47" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="48" max="48" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="49" max="49" style="7" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="50" max="50" style="9" width="24.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="7" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="7" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="6" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="6" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="6" width="16.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="6" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="6" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="6" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="6" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="6" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="6" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="6" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="6" width="22.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="6" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="6" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="6" width="18.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="6" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="6" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="6" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="50" max="50" style="7" width="24.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="73.5" customFormat="1" s="1">
@@ -1602,7 +1596,7 @@
       <c r="AW1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="4" t="s">
+      <c r="AX1" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1752,7 +1746,7 @@
       <c r="AW2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="AX2" s="4" t="s">
+      <c r="AX2" s="2" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1765,7 +1759,7 @@
         <v>97</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="5"/>
+      <c r="E3" s="4"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -1785,7 +1779,7 @@
       <c r="N3" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="O3" s="5" t="s">
         <v>103</v>
       </c>
       <c r="P3" s="2" t="s">

</xml_diff>